<commit_message>
GUI recherche FR et plus de resultats
</commit_message>
<xml_diff>
--- a/bibliotheque.xlsx
+++ b/bibliotheque.xlsx
@@ -166,7 +166,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>2</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="952500" cy="1428750"/>
@@ -177,6 +177,331 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -479,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,7 +817,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Date : 2026-08-02 16:52:11</t>
+          <t>Date : 2026-08-02 20:23:37</t>
         </is>
       </c>
     </row>
@@ -503,7 +828,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -521,30 +846,70 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Roman jeunesse</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>French language materials</t>
+          <t>Genre non repertorié</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Bande dessinée</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Fiction</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Young Adult Nonfiction</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Humor</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cuisine</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -559,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -641,67 +1006,578 @@
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3" ht="405" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Tintin au Congo</t>
+          <t>Le Seigneur des Anneaux T1 La fraternité de l'anneau</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>J.R.R. Tolkien</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>9782267051896</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Dans un paisible village du Comté, le jeune Frodo est sur le point de recevoir un cadeau qui changera sa vie à jamais : l’Anneau de Pouvoir. Forgé par Sauron au cœur de la Montagne du Feu, on croyait l’Anneau perdu depuis qu’un homme l’avait arraché au Seigneur des Ténèbres avant de le chasser hors du monde. À présent, de noirs présages s’étendent à nouveau sur la Terre du Milieu, les créatures maléfiques se multiplient et, dans les Montagnes de Brume, les Orques traquent les Nains. L’ennemi veut récupérer son bien afin de dominer le monde ; l’Œil de Sauron est désormais pointé sur le Comté. Heureusement Gandalf les a devancés. S’ils font vite, Frodo et lui parviendront peut-être à détruire l’Anneau à temps. Chef-d’œuvre de la fantasy, découverte d’un monde imaginaire, de sa géographie, de son histoire et de ses langues, mais aussi réflexion sur le pouvoir et la mort, Le Seigneur des Anneaux est sans équivalent par sa puissance d’évocation, son souffle et son ampleur. Cette traduction de Daniel Lauzon prend en compte la dernière version du texte anglais, les indications laissées par Tolkien à l’intention des traducteurs et les découvertes permises par les publications posthumes proposées par Christopher Tolkien. Ce volume contient 18 illustrations d’Alan Lee, ainsi que deux cartes en couleur de la Terre du Milieu et du Comté.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Les tribulations de Tintin au Congo</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Hergé</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>French language materials</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>1984</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>img non trouvé</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="405" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Le Seigneur des Anneaux T1 La fraternité de l'anneau</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>J.R.R. Tolkien</t>
-        </is>
-      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>Genre non repertorié</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>9782267051896</t>
+          <t>9782203192157</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Dans un paisible village du Comté, le jeune Frodo est sur le point de recevoir un cadeau qui changera sa vie à jamais : l’Anneau de Pouvoir. Forgé par Sauron au cœur de la Montagne du Feu, on croyait l’Anneau perdu depuis qu’un homme l’avait arraché au Seigneur des Ténèbres avant de le chasser hors du monde. À présent, de noirs présages s’étendent à nouveau sur la Terre du Milieu, les créatures maléfiques se multiplient et, dans les Montagnes de Brume, les Orques traquent les Nains. L’ennemi veut récupérer son bien afin de dominer le monde ; l’Œil de Sauron est désormais pointé sur le Comté. Heureusement Gandalf les a devancés. S’ils font vite, Frodo et lui parviendront peut-être à détruire l’Anneau à temps. Chef-d’œuvre de la fantasy, découverte d’un monde imaginaire, de sa géographie, de son histoire et de ses langues, mais aussi réflexion sur le pouvoir et la mort, Le Seigneur des Anneaux est sans équivalent par sa puissance d’évocation, son souffle et son ampleur. Cette traduction de Daniel Lauzon prend en compte la dernière version du texte anglais, les indications laissées par Tolkien à l’intention des traducteurs et les découvertes permises par les publications posthumes proposées par Christopher Tolkien. Ce volume contient 18 illustrations d’Alan Lee, ainsi que deux cartes en couleur de la Terre du Milieu et du Comté.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Description non repertorié</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>img non repertorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="180" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Harry Potter à L'école des Sorciers</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>J.K. Rowling</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>9781781101032</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Le jour de ses onze ans, Harry Potter, un orphelin élevé par un oncle et une tante qui le détestent, voit son existence bouleversée. Un géant vient le chercher pour l’emmener à Poudlard, une école de sorcellerie! Voler en balai, jeter des sorts, combattre les trolls : Harry Potter se révèle un sorcier doué. Mais un mystère entoure sa naissance et l’effroyable V..., le mage dont personne n’ose prononcer le nom. Amitié, surprises, dangers, scènes comiques, Harry découvre ses pouvoirs et la vie à Poudlard. Le premier tome des aventures du jeune héros vous ensorcelle aussitôt!</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="135" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Le Secret de La Licorne</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Hergé</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Young Adult Nonfiction</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>1943</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>9782203001107</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>En fouillant le grenier, le capitaine Haddock retrouve la trace de son ancêtre, le chevalier de Haddoque. Ce légendaire loup des mers s'est rendu célèbre par ses déboires avec le cruel pirate Rackham le Rouge. Un roman maritime de plus ? Certainement pas! Car le chevalier devient le dépositaire d'un fabuleux trésor. Pour Tintin, Haddock et une série de malfrats, il s'agit de le retrouver. Mais les pistes et les énigmes se multiplient.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="112.5" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Asterix - L'anniversaire d'Astérix et Obélix - n°34</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>René Goscinny</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Bande dessinée</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>9782864973065</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Pour le 50ème anniversaire de leur création, Albert Uderzo, offre à ses personnages l'hypothètique humanité de les faire vieillir...de 50 ans ! Saurez-vous reconnaitre vos personnages gaulois favoris parmi ce défilé hilarant de détournements et de caricatures ?</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="180" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Harry Potter et la Coupe de Feu</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>J.K. Rowling</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>9781781101063</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Harry Potter a quatorze ans et entre en quatrième année au collège de Poudlard. Une grande nouvelle attend Harry, Ron et Hermione à leur arrivée : la tenue d’un tournoi de magie exceptionnel entre les plus célèbres écoles de sorcellerie. Déjà les délégations étrangères font leur entrée. Harry se réjouit... Trop vite. Il va se trouver plongé au coeur des événements les plus dramatiques qu’il ait jamais eu à affronter. Dans ce quatrième tome bouleversant, drôle, fascinant, qui révèle la richesse des enjeux en cours, Harry Potter doitfaire face et relever d’immenses défis.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9" ht="405" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Harry Potter et l'ordre du Phénix</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Joanne Kathleen Rowling</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Genre non repertorié</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>9782070585212</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>J. K. Rowling est l'auteur des sept romans de la saga Harry Potter. Traduite en 79 langues, vendue à des millions d'exemplaires et adaptée en 8 films à succès par Warner Bros, cette saga est aujourd'hui un véritable phénomène littéraire et l'une des oeuvres les plus lues au monde. J. K Rowling a également signé trois ouvrages de la Bibliothèque de Poudlard publiés au profit d'organisations caritatives : "Les Contes de Beedle le Barde" pour sa propre association d'aide aux enfants, Lumos ; "Le Quidditch à travers les âges" et "Les Animaux fantastiques" pour les associations Comic Relief et Lumos. Elle a imaginé, avec l'auteur Jack Thorne et le metteur en scène John Tiffany, la pièce "Harry Potter et l'enfant maudit", dont les premières représentations ont eu lieu à Londres durant l'été 2016. On lui doit aussi des romans pour adultes : "Une place à prendre" et, sous le pseudonyme de Robert Galbraith, trois enquêtes du détective Cormoran Strike. En 2017, elle publie son premier scénario, "Les Animaux fantastiques" : le texte du film. La même année, J. K. Rowling a été nommée Companion of Honour par la reine d'Angleterre. Elle est la plus jeune personnalité à avoir reçu cette distinction, la plus haute du royaume. Son site et éditeur numérique, Pottermore, est la plateforme numérique du "Monde des Sorciers".</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>img non repertorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="300" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Miaouw</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Feliz Paludin</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Genre non repertorié</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>9798396015098</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Moustache et Biscuit sont deux chats qui aiment les enquêtes et qui n'ont pas froid aux yeux. Quand Madame Perle, une chatte persane, leur confie la mission de retrouver son collier volé par une bande de voyous, ils n'hésitent pas une seconde. Ils se lancent dans une aventure palpitante qui les mène sur une île aux pirates où ils découvrent un trésor maudit. En chemin, ils se font des amis, des ennemis, et trouvent l'amour. Ils apprennent aussi des secrets sur le passé des chats grâce à un livre rare qu'ils gagnent à un concours de chant. Mais attention, le danger les guette à chaque instant. Parviendront-ils à accomplir leur mission et à sauver le monde ? Découvrez-le dans cette histoire pleine de suspense et d'aventure, où les chats sont les héros ! Ce livre non conventionnel a été écrit pour un large public. Il s'adresse aussi bien aux humains, qu'ils soient enfants ou adultes, qu'aux félins. Ce livre est à la fois écrit en langue humaine et en langue chat.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Vous avez ma parole</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Jean-Marie Le Pen</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Genre non repertorié</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>9782912104120</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Description non repertorié</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>img non repertorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="112.5" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Current Biography</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Genre non repertorié</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>ISBN non repertorié</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Description non repertorié</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13" ht="165" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Jean-Pierre Coffe - Tome 3 - Les Recettes de fêtes inratables de Jean-Pierre Coffe</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Jack Domon</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Humor</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>9782822202343</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Apprendre en s'amusant pour réussir toutes les fêtes.Une chose est sûre avec Jean-Pierre Coffe: petits et grands vont pouvoir faire la fête! Noël, les anniversaires, Saint-Nicolas, Pâques, Epiphanie, Mardi gras, la fête des Mères et des Pères, toutes les occasions sont bonnes pour se régaler! Jean-Pierre Coffe vous invite à découvrir les recettes traditionnelles des régions de France et d'Europe pour les fêtes. Apprenez à préparer tous ces plats délicieux à partager avec votre famille et vos amis.Bon Appétit!</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14" ht="112.5" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>La boutique de Maman Chichigneux</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Jacqueline Verly</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>9782402182355</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Cet ouvrage est une réédition numérique d’un livre paru au XXe siècle, désormais indisponible dans son format d’origine.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15" ht="285" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>So French</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Dany Chouet</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Cuisine</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>9781743438404</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>From Dany's childhood in post-war France, to her migration to Australia and rise to culinary success - this is truly a book to devour! Acclaimed restaurateur Dany Chouet helped shape French cuisine in Australia throughout the 1970s, 80's and 90's through her successful restaurants Upstairs, Au Chabrol, Glenella and Cleopatra. Now back in south-west France, she and her partner are wooing international customers with gourmet tours and Dany's quintessential country cooking. In her first book, So French, Dany tells her fascinating life story which is interwoven with more than 60 timeless recipes and complemented by stunning images taken at her home in the south of France. From traditional garlic and onion soup to hearty salt cod and potato ragout and sweet nectarine and raspberry gratin, browsing through the pages of So French is sure to make your tastebuds tingle and your thoughts travel to provincial France.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16" ht="855" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>La guerre des Clans cycle I - Intégrale</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Erin Hunter</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>9782823861105</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Découvrez l'intégrale du premier cycle de L a Guerre des Clans en un seul ebook ! Tome 1 : Retour à l'état sauvage Depuis des générations, fidèles aux lois de leurs ancêtres, quatre clans de chats sauvages se partagent la forêt. Mais le Clan du Tonnerre court un grave danger, et les sinistres guerriers de l'Ombre sont de plus en plus puissants. En s'aventurant un jour dans les bois, Rusty, petit chat domestique, est loin de se douter qu'il deviendra bientôt le plus valaureux des guerriers... Tome 2 : À feu et à sang Au sein du Clan du Tonnerre, Coeur de Feu est devenu un valeureux guerrier. Une chance ! Il aura besoin de toutes ses forces pour déjouer les plans diaboliques de Griffe de Tigre qui cherche à lui nuire et à l'exclure de son clan. Sans parler des accidents et maladies qui s'abattent depuis quelques temps sur la tribu. Lorsque le clan voisin, celui du Vent, est chassé de ses terres, sa méfiance grandit encore. Déchiré, Coeur de Feu s'interroge : comment aider les autres quand on doit se défendre soi-même ? Tome 3 : Les Mystères de la forêt La tension est à son comble dans le Clan du Tonnerre : une terrible inondation s'abat sur la forêt et les alliances entre tribus changent sans cesse. Quant à Coeur de Feu, il continue d'enquêter sur la mort de Plume Rousse, l'ancien lieutenant du clan. Il ignore encore quelle sombre machination il va découvrir... Tome 4 : Avant la tempête Depuis la trahison de Griffe de Tigre, Cœur de Feu a pris de nouvelles responsabilités dans son clan. Mais le traître rôde toujours. Cœur de Feu se sent plus seul que jamais. Heureusement, l'amour qu'il porte à la belle Tempête de Sable le soulage du poids de ses lourdes tâches. Quand un danger terrible est sur le point de s'abattre sur la forêt, Cœur de Feu va devoir à nouveau prouver sa valeur. Tome 5 : Sur le sentier de la guerre Jamais Cœur de Feu n'aurait pensé devoir affronter tant d'épreuves ! Après l'incendie qui a ravagé la forêt, il se retrouve à la tête d'un clan affaibli. Et Étoile Bleue ne lui est d'aucun secours : la vieille meneuse n'est plus que l'ombre d'elle-même. Pourtant, un nouveau défi attend le jeune lieutenant : une meute de chiens sanguinaires rôde sur leur territoire. Dans la guerre impitoyable qui se prépare, pourra-t-il sauver les siens ? Tome 6 : Une sombre prophétie Etoile bleue est morte ! Ses guerriers sont sous le choc, et notamment Coeur de Feu, qui devient le meneur du clan. Le jeune guerrier reçoit alors dans son sommeil une prophétie étrange et effrayante : des temps obscurs se profilent pour lui et les siens. Au même moment, Etoile du Tigre, leur ennemi juré, fomente un nouveau complot. Pour conquérir le pouvoir absolu, il est prêt à pactiser avec une horde de chats impitoyables. Jamais l'équilibre fragile de la forêt n'a été si menacé...</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17" ht="165" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>La guerre des clans, Cycle VI - Tome 6 Au coeur de la tourmente</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Erin Hunter</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>9782823886993</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Poursuivez l'aventure du sixième cycle de La guerre des Clans ! Le Clan de l'Ombre est de retour et il souhaite récupérer l'intégralité de son ancien territoire, aujourd'hui en partie occupé par le Clan du Ciel. Mais trouver un accord se révèle difficile. Car si le premier a besoin de plus d'espace, le second ne peut se priver du gibier de ses terres... Les tensions s'enflamment jusqu'à un point de rupture explosif : la place de chacun des clans risque d'être remise en question une fois pour toutes !</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18" ht="180" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>La guerre des clans cycle III Le pouvoir des étoiles - tome 1 Vision</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Erin Hunter</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>9782266230490</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>La paix entre les Clans est-elle vraiment rétablie ? Tenaillé par la faim, le clan de l'Ombre tente d'agrandir son territoire et défie ses voisins. Étoile de Feu entend alors en rêve une nouvelle prophétie : " Ils seront trois, parents de tes parents, à détenir le pouvoir des Étoiles entre leurs griffes. " S'agit-il des petits de Griffe de Ronce, son lieutenant ? Petit Houx, Petit Lion et Petit Geai sortent à peine de la pouponnière. Pourtant la menace gronde, et pour la survie de leur clan ils devront se battre aussi vaillamment que les meilleurs guerriers.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19" ht="112.5" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>La guerre des Clans version illustrée cycle II - tome 3</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Erin Hunter</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Roman jeunesse</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>9782823818697</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Après avoir vaincu le Clan du Sang, Nuage de Jais et Gerboise sont prêts à reconquérir leur ferme. L'aide du Clan du Tonnerre suffira-t-elle à chasser la bande de chats sauvages qui s'y est établie ? Les deux amis devront trouver le courage de se battre en guerriers, sous peine de perdre à jamais leur territoire...</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>